<commit_message>
rm glc from fluxalilm 291c83cdd60a19dc326fdda9620071005b585a66
</commit_message>
<xml_diff>
--- a/nr-add-lipids/ig/StructureDefinition-mesures-bundle-flux-alimentation.xlsx
+++ b/nr-add-lipids/ig/StructureDefinition-mesures-bundle-flux-alimentation.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-27T13:15:18+00:00</t>
+    <t>2025-03-27T14:27:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -880,7 +880,7 @@
 MeasurementResultsTests</t>
   </si>
   <si>
-    <t xml:space="preserve">Observation {https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-bmi|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-bodyheight|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-body-temperature|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-body-weight|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-bp|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-heartrate|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-observation-glucose|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-observation-head-circumference|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-observation-pain-severity|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-observation-steps-by-day|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-observation-waist-circumference|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-oxygen-sat}
+    <t xml:space="preserve">Observation {https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-bmi|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-bodyheight|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-body-temperature|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-body-weight|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-bp|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-heartrate|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-observation-head-circumference|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-observation-pain-severity|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-observation-steps-by-day|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-observation-waist-circumference|https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-fr-observation-oxygen-sat}
 </t>
   </si>
   <si>
@@ -11014,7 +11014,7 @@
         <v>88</v>
       </c>
       <c r="K85" t="s" s="2">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="L85" t="s" s="2">
         <v>186</v>

</xml_diff>